<commit_message>
Daily MPR update | 12-02-2026
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
+++ b/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiwar\OneDrive\Desktop\New folder (3)\TH-PROJECT-NOTEBOOK\MPR\Role wise\Android Developer\Feb'26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F709D768-AF82-4994-AB33-E35A697A3F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1CDE9E-331E-449F-B5F7-43B8A86CF8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feb 2026" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="43">
   <si>
     <t>SR#</t>
   </si>
@@ -55,13 +55,121 @@
   </si>
   <si>
     <t>Comments</t>
+  </si>
+  <si>
+    <t>Attended Power BI team meeting – require discussion for new dashboard</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>Power Bi</t>
+  </si>
+  <si>
+    <t>2nd feb</t>
+  </si>
+  <si>
+    <t>Akash Tiwari</t>
+  </si>
+  <si>
+    <t>Discussed KPIs, data sources and visualization standards</t>
+  </si>
+  <si>
+    <t>3rd feb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enterprise app presentation - SIDC training  center </t>
+  </si>
+  <si>
+    <t xml:space="preserve">completed </t>
+  </si>
+  <si>
+    <t>Enterprise sakhi app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">whole day training 2 batch </t>
+  </si>
+  <si>
+    <t>Power BI stakeholder meeting – report enhancement planning</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Power BI</t>
+  </si>
+  <si>
+    <t>4th feb</t>
+  </si>
+  <si>
+    <t>inalized report structure and filter requirements</t>
+  </si>
+  <si>
+    <t>Worked on TMS PoC documentation , workflow and module descriptions</t>
+  </si>
+  <si>
+    <t>TMS</t>
+  </si>
+  <si>
+    <t>5th feb</t>
+  </si>
+  <si>
+    <t>Documented user roles and training lifecycle flow</t>
+  </si>
+  <si>
+    <t>6th feb</t>
+  </si>
+  <si>
+    <t>7th feb</t>
+  </si>
+  <si>
+    <t>Finalized report structure and filter requirements</t>
+  </si>
+  <si>
+    <t>Incorporated feedback and refined functional sections</t>
+  </si>
+  <si>
+    <t>8th feb</t>
+  </si>
+  <si>
+    <t>Final Review of Power BI Parameter and Sources meeting</t>
+  </si>
+  <si>
+    <t>9th feb</t>
+  </si>
+  <si>
+    <t>Verified technical and functional accuracy with team</t>
+  </si>
+  <si>
+    <t>Worked on TMS UI pages , Created pages on parameters</t>
+  </si>
+  <si>
+    <t>Creation of UI pages in software</t>
+  </si>
+  <si>
+    <t>10th feb</t>
+  </si>
+  <si>
+    <t>Continued TMS PoC documentation and internal review</t>
+  </si>
+  <si>
+    <t>Final review of POC TMS documents and summary preparation</t>
+  </si>
+  <si>
+    <t>11th feb</t>
+  </si>
+  <si>
+    <t>Consolidated the document and shared final version</t>
+  </si>
+  <si>
+    <t>Sunday</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +198,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -105,7 +219,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -128,26 +242,129 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,51 +646,369 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="42.140625" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" customWidth="1"/>
     <col min="5" max="5" width="14.5703125" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="B2" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily MPR update | 24-02-2026
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
+++ b/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiwar\OneDrive\Desktop\New folder (3)\TH-PROJECT-NOTEBOOK\MPR\Role wise\Android Developer\Feb'26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1CDE9E-331E-449F-B5F7-43B8A86CF8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF3CBAE-13ED-4937-A859-CF2BB8F44A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="78">
   <si>
     <t>SR#</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Incorporated feedback and refined functional sections</t>
   </si>
   <si>
-    <t>8th feb</t>
-  </si>
-  <si>
     <t>Final Review of Power BI Parameter and Sources meeting</t>
   </si>
   <si>
@@ -163,6 +160,114 @@
   </si>
   <si>
     <t>Sunday</t>
+  </si>
+  <si>
+    <t>Worked on Power BI team meeting – dashboard requirement discussion</t>
+  </si>
+  <si>
+    <t>12th feb</t>
+  </si>
+  <si>
+    <t>Discussed new KPIs and report enhancement requirements</t>
+  </si>
+  <si>
+    <t>Prepared MOM and documentation of discussed Power BI report changes</t>
+  </si>
+  <si>
+    <t>Shared meeting summary and action points with team</t>
+  </si>
+  <si>
+    <t>13th feb</t>
+  </si>
+  <si>
+    <t>SUNDAY</t>
+  </si>
+  <si>
+    <t>Cross-team coordination for TMS and Power BI documentation validation</t>
+  </si>
+  <si>
+    <t>TMS / Power BI</t>
+  </si>
+  <si>
+    <t>15th feb</t>
+  </si>
+  <si>
+    <t>Verified functional accuracy with technical team</t>
+  </si>
+  <si>
+    <t>16th feb</t>
+  </si>
+  <si>
+    <t>Worked on POC of EP Sakhi – requirement understanding and workflow analysis</t>
+  </si>
+  <si>
+    <t>EP Sakhi</t>
+  </si>
+  <si>
+    <t>17th Feb</t>
+  </si>
+  <si>
+    <t>Reviewed existing modules and documented functional flow</t>
+  </si>
+  <si>
+    <t>Continued POC development &amp; documentation of EP Sakhi modules</t>
+  </si>
+  <si>
+    <t>Ep SAAKHI</t>
+  </si>
+  <si>
+    <t>18th Feb</t>
+  </si>
+  <si>
+    <t>Prepared module-wise documentation and noted improvement points</t>
+  </si>
+  <si>
+    <t>Worked on BMM, DMM, SMM Login Page development</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Web Application</t>
+  </si>
+  <si>
+    <t>19th Feb</t>
+  </si>
+  <si>
+    <t>Implemented role-based login structure and basic validation logic</t>
+  </si>
+  <si>
+    <t>8th Feb</t>
+  </si>
+  <si>
+    <t>14th Feb</t>
+  </si>
+  <si>
+    <t>Integrated SHG member data fetching after login</t>
+  </si>
+  <si>
+    <t>20th Feb</t>
+  </si>
+  <si>
+    <t>Connected API for fetching SHG member list and handled role-wise data display</t>
+  </si>
+  <si>
+    <t>21st Feb</t>
+  </si>
+  <si>
+    <t>On leave due to Fever</t>
+  </si>
+  <si>
+    <t>On leave due to high fever</t>
+  </si>
+  <si>
+    <t>Prepared Change Request document for TMS and EP Sakhi and submitted to department</t>
+  </si>
+  <si>
+    <t>TMS / EP Sakhi</t>
+  </si>
+  <si>
+    <t>23rd Feb</t>
+  </si>
+  <si>
+    <t>Drafted detailed CR document including description, scope impact, and justification; shared with concerned department for review</t>
   </si>
 </sst>
 </file>
@@ -219,7 +324,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -305,11 +410,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -365,6 +481,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -646,7 +782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.140625" customWidth="1"/>
@@ -656,7 +792,7 @@
     <col min="7" max="7" width="25.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -679,12 +815,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -692,7 +828,7 @@
       <c r="F2" s="17"/>
       <c r="G2" s="18"/>
     </row>
-    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -715,7 +851,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -738,7 +874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -763,7 +899,7 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -788,7 +924,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -811,81 +947,81 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="23">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C8" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="F8" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="21" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>35</v>
+      <c r="B9" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="13">
+        <v>9</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="C10" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="E10" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>19</v>
@@ -894,7 +1030,7 @@
         <v>24</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>11</v>
@@ -903,12 +1039,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>19</v>
@@ -917,95 +1053,314 @@
         <v>24</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
+    </row>
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>13</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>15</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="26">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="26">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+    </row>
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="8">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Daily DPR Update | 24-02-26
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
+++ b/MPR/Role wise/Android Developer/Feb'26/Individual_MPR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiwar\OneDrive\Desktop\New folder (3)\TH-PROJECT-NOTEBOOK\MPR\Role wise\Android Developer\Feb'26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\TH-PROJECT-NOTEBOOK\MPR\Role wise\Android Developer\Feb'26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF3CBAE-13ED-4937-A859-CF2BB8F44A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9D5219-E452-4034-9CB9-37EC84F5A6C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feb 2026" sheetId="1" r:id="rId1"/>
@@ -258,9 +258,6 @@
     <t>On leave due to high fever</t>
   </si>
   <si>
-    <t>Prepared Change Request document for TMS and EP Sakhi and submitted to department</t>
-  </si>
-  <si>
     <t>TMS / EP Sakhi</t>
   </si>
   <si>
@@ -268,6 +265,9 @@
   </si>
   <si>
     <t>Drafted detailed CR document including description, scope impact, and justification; shared with concerned department for review</t>
+  </si>
+  <si>
+    <t>Prepared Change Request document for TMS and submitted to department</t>
   </si>
 </sst>
 </file>
@@ -1335,22 +1335,22 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>